<commit_message>
updating all scenario files
</commit_message>
<xml_diff>
--- a/Outputs/Scenarios/PtX_demand_AT_Electrification.xlsx
+++ b/Outputs/Scenarios/PtX_demand_AT_Electrification.xlsx
@@ -1592,7 +1592,7 @@
         <v>0</v>
       </c>
       <c r="K31" t="n">
-        <v>5.507271038521231e-05</v>
+        <v>5.50727103852123e-05</v>
       </c>
     </row>
     <row r="32">
@@ -1999,7 +1999,7 @@
         <v>0.0003228682160306722</v>
       </c>
       <c r="K42" t="n">
-        <v>5.507271038521231e-05</v>
+        <v>5.50727103852123e-05</v>
       </c>
     </row>
     <row r="43">

</xml_diff>